<commit_message>
Dados atualizados em 26/10/2026 09:13
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA9C3B2-2795-4729-A33F-6198F0EE3186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA2C6A9-6DF1-4D5F-A4AE-B60DE4D2A135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -42,14 +42,13 @@
     <metadataType name="XLMDX" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
-  <metadataStrings count="5">
+  <metadataStrings count="4">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
     <s v="{[Intervalo 2].[PRODUTO].&amp;[MIST PAO DA FAZENDA VIAPANE 10KG]}"/>
     <s v="{[Intervalo 2].[DES_TIPO_OPERACAO].&amp;[VENDA],[Intervalo 2].[DES_TIPO_OPERACAO].&amp;[VENDA SAT]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-10-09T00:00:00]}"/>
   </metadataStrings>
-  <mdxMetadata count="4">
+  <mdxMetadata count="3">
     <mdx n="0" f="s">
       <ms ns="1" c="0"/>
     </mdx>
@@ -58,9 +57,6 @@
     </mdx>
     <mdx n="0" f="s">
       <ms ns="3" c="0"/>
-    </mdx>
-    <mdx n="0" f="s">
-      <ms ns="4" c="0"/>
     </mdx>
   </mdxMetadata>
   <futureMetadata name="XLDAPR" count="1">
@@ -77,7 +73,7 @@
       <rc t="2" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="4">
+  <valueMetadata count="3">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -86,9 +82,6 @@
     </bk>
     <bk>
       <rc t="1" v="2"/>
-    </bk>
-    <bk>
-      <rc t="1" v="3"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -2510,8 +2503,8 @@
           <cell r="K1" t="str">
             <v>POSITIVACAO PAO DA FAZENDA</v>
           </cell>
-          <cell r="L1">
-            <v>3</v>
+          <cell r="L1" t="e">
+            <v>#VALUE!</v>
           </cell>
           <cell r="M1">
             <v>0</v>
@@ -2527,8 +2520,8 @@
           <cell r="H2" t="str">
             <v>DATA</v>
           </cell>
-          <cell r="I2" t="str" vm="4">
-            <v>09/10/2026</v>
+          <cell r="I2" t="str" vm="1">
+            <v>All</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -2570,30 +2563,30 @@
         </row>
         <row r="5">
           <cell r="E5" t="str">
-            <v>(vazio)</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>175.08999999999997</v>
+            <v>48786.559999999998</v>
           </cell>
           <cell r="H5" t="str">
-            <v>(vazio)</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>175.08999999999997</v>
+            <v>48786.559999999998</v>
           </cell>
         </row>
         <row r="6">
           <cell r="E6" t="str">
-            <v>CAMPINAS</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>19043.580000000002</v>
+            <v>272619.34999999963</v>
           </cell>
           <cell r="H6" t="str">
-            <v>CAMPINAS</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>1270.82</v>
+            <v>272619.34999999963</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -2604,16 +2597,16 @@
         </row>
         <row r="7">
           <cell r="E7" t="str">
-            <v>CENTRO</v>
+            <v>ECOMMERCE</v>
           </cell>
           <cell r="F7">
-            <v>117001.94999999997</v>
+            <v>869.6400000000001</v>
           </cell>
           <cell r="H7" t="str">
-            <v>CENTRO</v>
+            <v>ECOMMERCE</v>
           </cell>
           <cell r="I7">
-            <v>11533.52</v>
+            <v>869.6400000000001</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -2627,16 +2620,16 @@
         </row>
         <row r="8">
           <cell r="E8" t="str">
-            <v>ECOMMERCE</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="F8">
-            <v>75.12</v>
+            <v>62260.590000000026</v>
           </cell>
           <cell r="H8" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I8">
-            <v>4577.72</v>
+            <v>62260.590000000026</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
@@ -2650,16 +2643,16 @@
         </row>
         <row r="9">
           <cell r="E9" t="str">
-            <v>IATAGAM JUNIOR</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="F9">
-            <v>324.10000000000002</v>
+            <v>203747.14999999964</v>
           </cell>
           <cell r="H9" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I9">
-            <v>10562.029999999999</v>
+            <v>203747.14999999964</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
@@ -2673,16 +2666,16 @@
         </row>
         <row r="10">
           <cell r="E10" t="str">
-            <v>INDAIATUBA</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="F10">
-            <v>25865.750000000011</v>
+            <v>71931.839999999822</v>
           </cell>
           <cell r="H10" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="I10">
-            <v>2244.54</v>
+            <v>71931.839999999822</v>
           </cell>
           <cell r="K10" t="str">
             <v>INTERLAGOS</v>
@@ -2696,16 +2689,16 @@
         </row>
         <row r="11">
           <cell r="E11" t="str">
-            <v>INTERLAGOS</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="F11">
-            <v>87405.690000000031</v>
+            <v>194941.35</v>
           </cell>
           <cell r="H11" t="str">
             <v>KEY ABC</v>
           </cell>
           <cell r="I11">
-            <v>5041.5</v>
+            <v>194941.35</v>
           </cell>
           <cell r="K11" t="str">
             <v>JUNDIAI</v>
@@ -2719,16 +2712,16 @@
         </row>
         <row r="12">
           <cell r="E12" t="str">
-            <v>JUNDIAI</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="F12">
-            <v>28099.500000000029</v>
+            <v>350628.99999999953</v>
           </cell>
           <cell r="H12" t="str">
             <v>KEY CASA</v>
           </cell>
           <cell r="I12">
-            <v>7043</v>
+            <v>350628.99999999953</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE MOOCA</v>
@@ -2742,16 +2735,16 @@
         </row>
         <row r="13">
           <cell r="E13" t="str">
-            <v>KEY ABC</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="F13">
-            <v>90046.700000000012</v>
+            <v>560129.58000000042</v>
           </cell>
           <cell r="H13" t="str">
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="I13">
-            <v>66439.199999999997</v>
+            <v>560129.58000000042</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE PENHA</v>
@@ -2765,16 +2758,16 @@
         </row>
         <row r="14">
           <cell r="E14" t="str">
-            <v>KEY CASA</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="F14">
-            <v>104355.99000000003</v>
+            <v>45062.200000000004</v>
           </cell>
           <cell r="H14" t="str">
             <v>KEY SJC</v>
           </cell>
           <cell r="I14">
-            <v>3909.2</v>
+            <v>45062.200000000004</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE TATUAPE</v>
@@ -2788,16 +2781,16 @@
         </row>
         <row r="15">
           <cell r="E15" t="str">
-            <v>KEY INTERIOR</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="F15">
-            <v>284976.00000000006</v>
+            <v>288574.25999999995</v>
           </cell>
           <cell r="H15" t="str">
             <v>KEY SP</v>
           </cell>
           <cell r="I15">
-            <v>11131.059999999998</v>
+            <v>288574.25999999995</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
@@ -2811,16 +2804,16 @@
         </row>
         <row r="16">
           <cell r="E16" t="str">
-            <v>KEY SJC</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="F16">
-            <v>10406.4</v>
+            <v>334703.23000000004</v>
           </cell>
           <cell r="H16" t="str">
             <v>KEY ZL</v>
           </cell>
           <cell r="I16">
-            <v>3757.1</v>
+            <v>334703.23000000004</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
@@ -2834,16 +2827,16 @@
         </row>
         <row r="17">
           <cell r="E17" t="str">
-            <v>KEY SP</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="F17">
-            <v>76109.040000000023</v>
+            <v>148229.4349999995</v>
           </cell>
           <cell r="H17" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I17">
-            <v>988.43000000000006</v>
+            <v>148229.4349999995</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
@@ -2857,39 +2850,39 @@
         </row>
         <row r="18">
           <cell r="E18" t="str">
-            <v>KEY ZL</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="F18">
-            <v>112434.5800000001</v>
+            <v>130217.75999999982</v>
           </cell>
           <cell r="H18" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I18">
-            <v>4973.12</v>
+            <v>130217.75999999982</v>
           </cell>
           <cell r="K18" t="str">
             <v>SBC</v>
           </cell>
           <cell r="L18">
-            <v>10</v>
+            <v>9</v>
           </cell>
           <cell r="M18">
-            <v>10</v>
+            <v>9</v>
           </cell>
         </row>
         <row r="19">
           <cell r="E19" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F19">
-            <v>56477.170000000086</v>
+            <v>122031.32999999971</v>
           </cell>
           <cell r="H19" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I19">
-            <v>1402.54</v>
+            <v>122031.32999999971</v>
           </cell>
           <cell r="K19" t="str">
             <v>SJC</v>
@@ -2903,16 +2896,16 @@
         </row>
         <row r="20">
           <cell r="E20" t="str">
-            <v>LESTE PENHA</v>
+            <v>MOGI</v>
           </cell>
           <cell r="F20">
-            <v>48456.710000000006</v>
+            <v>45154.940000000046</v>
           </cell>
           <cell r="H20" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="I20">
-            <v>2549.5500000000002</v>
+            <v>45154.940000000046</v>
           </cell>
           <cell r="K20" t="str">
             <v>SJC/VALE</v>
@@ -2926,123 +2919,123 @@
         </row>
         <row r="21">
           <cell r="E21" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>NORTE</v>
           </cell>
           <cell r="F21">
-            <v>32493.730000000003</v>
+            <v>211937.01999999859</v>
           </cell>
           <cell r="H21" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="I21">
-            <v>5135.0499999999984</v>
+            <v>211937.01999999859</v>
           </cell>
           <cell r="K21" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="L21">
-            <v>100</v>
+            <v>99</v>
           </cell>
           <cell r="M21">
-            <v>100</v>
+            <v>99</v>
           </cell>
         </row>
         <row r="22">
           <cell r="E22" t="str">
-            <v>MOGI</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="F22">
-            <v>18272.769999999997</v>
+            <v>251412.51500000042</v>
           </cell>
           <cell r="H22" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="I22">
-            <v>13963.489999999998</v>
+            <v>251412.51500000042</v>
           </cell>
         </row>
         <row r="23">
           <cell r="E23" t="str">
-            <v>NORTE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="F23">
-            <v>81243.350000000093</v>
+            <v>107918.3099999995</v>
           </cell>
           <cell r="H23" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I23">
-            <v>2919.1</v>
+            <v>107918.3099999995</v>
           </cell>
         </row>
         <row r="24">
           <cell r="E24" t="str">
-            <v>OSASCO</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="F24">
-            <v>114216.91000000018</v>
+            <v>135944.54999999996</v>
           </cell>
           <cell r="H24" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I24">
-            <v>2159.1999999999998</v>
+            <v>135944.54999999996</v>
           </cell>
         </row>
         <row r="25">
           <cell r="E25" t="str">
-            <v>PIRITUBA</v>
+            <v>SBC</v>
           </cell>
           <cell r="F25">
-            <v>44023.619999999988</v>
+            <v>215409.78999999963</v>
           </cell>
           <cell r="H25" t="str">
             <v>SBC</v>
           </cell>
           <cell r="I25">
-            <v>15594.409999999996</v>
+            <v>215409.78999999963</v>
           </cell>
         </row>
         <row r="26">
           <cell r="E26" t="str">
-            <v>SANTO ANDRE</v>
+            <v>SJC</v>
           </cell>
           <cell r="F26">
-            <v>53099.140000000007</v>
+            <v>59228.230000000018</v>
           </cell>
           <cell r="H26" t="str">
             <v>SJC</v>
           </cell>
           <cell r="I26">
-            <v>5642.74</v>
+            <v>59228.230000000018</v>
           </cell>
         </row>
         <row r="27">
           <cell r="E27" t="str">
-            <v>SBC</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="F27">
-            <v>89009.680000000051</v>
+            <v>39507.460000000057</v>
           </cell>
           <cell r="H27" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="I27">
-            <v>1484.7000000000003</v>
+            <v>39507.460000000057</v>
           </cell>
         </row>
         <row r="28">
           <cell r="E28" t="str">
-            <v>SJC</v>
+            <v>VENDA B2E</v>
           </cell>
           <cell r="F28">
-            <v>27951.950000000019</v>
+            <v>495.46</v>
           </cell>
           <cell r="H28" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>VENDA B2E</v>
           </cell>
           <cell r="I28">
-            <v>2619.7000000000003</v>
+            <v>495.46</v>
           </cell>
           <cell r="K28" t="str">
             <v>POSITIVAÇÃO GERAL</v>
@@ -3050,16 +3043,16 @@
         </row>
         <row r="29">
           <cell r="E29" t="str">
-            <v>SJC/VALE</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F29">
-            <v>15939.879999999988</v>
+            <v>58769.760000000009</v>
           </cell>
           <cell r="H29" t="str">
-            <v>Total Geral</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I29">
-            <v>187116.80999999997</v>
+            <v>58769.760000000009</v>
           </cell>
           <cell r="K29" t="str">
             <v>DATA</v>
@@ -3070,24 +3063,22 @@
         </row>
         <row r="30">
           <cell r="E30" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="F30">
-            <v>24446.020000000004</v>
+            <v>3960511.3099999744</v>
+          </cell>
+          <cell r="H30" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I30">
+            <v>3960511.3099999744</v>
           </cell>
           <cell r="K30" t="str">
             <v>DES_TIPO_OPERACAO</v>
           </cell>
           <cell r="L30" t="str" vm="3">
             <v>(Vários itens)</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="E31" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="F31">
-            <v>1561950.4200000046</v>
           </cell>
         </row>
         <row r="32">
@@ -3117,10 +3108,10 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="L34">
-            <v>53</v>
+            <v>68</v>
           </cell>
           <cell r="M34">
-            <v>53</v>
+            <v>68</v>
           </cell>
         </row>
         <row r="35">
@@ -3128,10 +3119,10 @@
             <v>Total Geral</v>
           </cell>
           <cell r="L35">
-            <v>53</v>
+            <v>68</v>
           </cell>
           <cell r="M35">
-            <v>53</v>
+            <v>68</v>
           </cell>
         </row>
         <row r="39">
@@ -3139,7 +3130,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="B39">
-            <v>5750</v>
+            <v>5870</v>
           </cell>
         </row>
         <row r="40">
@@ -3147,7 +3138,7 @@
             <v>CENTRO</v>
           </cell>
           <cell r="B40">
-            <v>31000</v>
+            <v>32000</v>
           </cell>
         </row>
         <row r="41">
@@ -3155,7 +3146,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="B41">
-            <v>15530</v>
+            <v>15850</v>
           </cell>
         </row>
         <row r="42">
@@ -3163,7 +3154,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="B42">
-            <v>25000</v>
+            <v>24730</v>
           </cell>
         </row>
         <row r="43">
@@ -3171,7 +3162,7 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="B43">
-            <v>5700</v>
+            <v>5820</v>
           </cell>
         </row>
         <row r="44">
@@ -3179,7 +3170,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="B44">
-            <v>19890</v>
+            <v>17000</v>
           </cell>
         </row>
         <row r="45">
@@ -3195,7 +3186,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="B46">
-            <v>19770</v>
+            <v>20630</v>
           </cell>
         </row>
         <row r="47">
@@ -3203,7 +3194,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="B47">
-            <v>10110</v>
+            <v>9790</v>
           </cell>
           <cell r="P47" t="str">
             <v>Soma de TOTAL</v>
@@ -3222,7 +3213,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="B49">
-            <v>28000</v>
+            <v>28040</v>
           </cell>
         </row>
         <row r="50">
@@ -3230,7 +3221,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="B50">
-            <v>14510</v>
+            <v>14810</v>
           </cell>
         </row>
         <row r="51">
@@ -3238,7 +3229,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="B51">
-            <v>19620</v>
+            <v>18000</v>
           </cell>
         </row>
         <row r="52">
@@ -3246,7 +3237,7 @@
             <v>SBC</v>
           </cell>
           <cell r="B52">
-            <v>24000</v>
+            <v>25000</v>
           </cell>
         </row>
         <row r="53">
@@ -3254,7 +3245,7 @@
             <v>SJC</v>
           </cell>
           <cell r="B53">
-            <v>15300</v>
+            <v>15790</v>
           </cell>
         </row>
         <row r="54">
@@ -3262,7 +3253,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="B54">
-            <v>8980</v>
+            <v>10060</v>
           </cell>
         </row>
         <row r="55">
@@ -3270,7 +3261,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="B55">
-            <v>10850</v>
+            <v>11080</v>
           </cell>
         </row>
         <row r="63">
@@ -3441,13 +3432,13 @@
             <v>14</v>
           </cell>
           <cell r="F136">
-            <v>3</v>
+            <v>0</v>
           </cell>
           <cell r="H136" t="str">
             <v>D</v>
           </cell>
           <cell r="I136">
-            <v>11</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="137">
@@ -3455,13 +3446,13 @@
             <v>36</v>
           </cell>
           <cell r="F137">
-            <v>53</v>
+            <v>0</v>
           </cell>
           <cell r="H137" t="str">
-            <v>C</v>
+            <v>D</v>
           </cell>
           <cell r="I137">
-            <v>3</v>
+            <v>36</v>
           </cell>
         </row>
         <row r="138">
@@ -3469,13 +3460,13 @@
             <v>14</v>
           </cell>
           <cell r="F138">
-            <v>5</v>
+            <v>0</v>
           </cell>
           <cell r="H138" t="str">
             <v>D</v>
           </cell>
           <cell r="I138">
-            <v>9</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="139">
@@ -3483,13 +3474,13 @@
             <v>14</v>
           </cell>
           <cell r="F139">
-            <v>21</v>
+            <v>0</v>
           </cell>
           <cell r="H139" t="str">
-            <v>C</v>
+            <v>D</v>
           </cell>
           <cell r="I139">
-            <v>3.5</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="140">
@@ -3497,13 +3488,13 @@
             <v>14</v>
           </cell>
           <cell r="F140">
+            <v>0</v>
+          </cell>
+          <cell r="H140" t="str">
+            <v>D</v>
+          </cell>
+          <cell r="I140">
             <v>14</v>
-          </cell>
-          <cell r="H140" t="str">
-            <v>C</v>
-          </cell>
-          <cell r="I140">
-            <v>10.5</v>
           </cell>
         </row>
         <row r="141">
@@ -3511,13 +3502,13 @@
             <v>14</v>
           </cell>
           <cell r="F141">
-            <v>12</v>
+            <v>0</v>
           </cell>
           <cell r="H141" t="str">
             <v>D</v>
           </cell>
           <cell r="I141">
-            <v>2</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="142">
@@ -3525,13 +3516,13 @@
             <v>14</v>
           </cell>
           <cell r="F142">
-            <v>7</v>
+            <v>0</v>
           </cell>
           <cell r="H142" t="str">
             <v>D</v>
           </cell>
           <cell r="I142">
-            <v>7</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="143">
@@ -3567,13 +3558,13 @@
             <v>14</v>
           </cell>
           <cell r="F145">
-            <v>3</v>
+            <v>0</v>
           </cell>
           <cell r="H145" t="str">
             <v>D</v>
           </cell>
           <cell r="I145">
-            <v>11</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="146">
@@ -3581,13 +3572,13 @@
             <v>14</v>
           </cell>
           <cell r="F146">
-            <v>4</v>
+            <v>0</v>
           </cell>
           <cell r="H146" t="str">
             <v>D</v>
           </cell>
           <cell r="I146">
-            <v>10</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="147">
@@ -3609,13 +3600,13 @@
             <v>14</v>
           </cell>
           <cell r="F148">
-            <v>3</v>
+            <v>0</v>
           </cell>
           <cell r="H148" t="str">
             <v>D</v>
           </cell>
           <cell r="I148">
-            <v>11</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="149">
@@ -3623,13 +3614,13 @@
             <v>14</v>
           </cell>
           <cell r="F149">
-            <v>6</v>
+            <v>0</v>
           </cell>
           <cell r="H149" t="str">
             <v>D</v>
           </cell>
           <cell r="I149">
-            <v>8</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="150">
@@ -3637,13 +3628,13 @@
             <v>14</v>
           </cell>
           <cell r="F150">
-            <v>9</v>
+            <v>0</v>
           </cell>
           <cell r="H150" t="str">
             <v>D</v>
           </cell>
           <cell r="I150">
-            <v>5</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="151">
@@ -3651,13 +3642,13 @@
             <v>14</v>
           </cell>
           <cell r="F151">
-            <v>10</v>
+            <v>0</v>
           </cell>
           <cell r="H151" t="str">
             <v>D</v>
           </cell>
           <cell r="I151">
-            <v>4</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="152">
@@ -3679,13 +3670,13 @@
             <v>14</v>
           </cell>
           <cell r="F153">
-            <v>3</v>
+            <v>0</v>
           </cell>
           <cell r="H153" t="str">
             <v>D</v>
           </cell>
           <cell r="I153">
-            <v>11</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="154">
@@ -3693,10 +3684,10 @@
             <v>260</v>
           </cell>
           <cell r="F154">
-            <v>153</v>
+            <v>0</v>
           </cell>
           <cell r="I154">
-            <v>148</v>
+            <v>260</v>
           </cell>
         </row>
         <row r="158">
@@ -3718,13 +3709,13 @@
             <v>39600</v>
           </cell>
           <cell r="F159">
-            <v>27951.950000000019</v>
+            <v>59228.230000000018</v>
           </cell>
           <cell r="H159" t="str">
-            <v>D</v>
+            <v>C</v>
           </cell>
           <cell r="I159">
-            <v>11648.049999999981</v>
+            <v>2371.769999999975</v>
           </cell>
         </row>
         <row r="160">
@@ -3732,13 +3723,13 @@
             <v>35550</v>
           </cell>
           <cell r="F160">
-            <v>24446.020000000004</v>
+            <v>58769.760000000009</v>
           </cell>
           <cell r="H160" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I160">
-            <v>11103.979999999996</v>
+            <v>8380.2399999999907</v>
           </cell>
         </row>
         <row r="161">
@@ -3746,13 +3737,13 @@
             <v>155250</v>
           </cell>
           <cell r="F161">
-            <v>117001.94999999997</v>
+            <v>272619.34999999963</v>
           </cell>
           <cell r="H161" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I161">
-            <v>38248.050000000032</v>
+            <v>20630.650000000373</v>
           </cell>
         </row>
         <row r="162">
@@ -3760,13 +3751,13 @@
             <v>149175</v>
           </cell>
           <cell r="F162">
-            <v>114216.91000000018</v>
+            <v>251412.51500000042</v>
           </cell>
           <cell r="H162" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I162">
-            <v>34958.089999999822</v>
+            <v>30362.484999999579</v>
           </cell>
         </row>
         <row r="163">
@@ -3774,13 +3765,13 @@
             <v>126450</v>
           </cell>
           <cell r="F163">
-            <v>87405.690000000031</v>
+            <v>203747.14999999964</v>
           </cell>
           <cell r="H163" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I163">
-            <v>39044.309999999969</v>
+            <v>35102.850000000355</v>
           </cell>
         </row>
         <row r="164">
@@ -3788,13 +3779,13 @@
             <v>92700</v>
           </cell>
           <cell r="F164">
-            <v>56477.170000000086</v>
+            <v>148229.4349999995</v>
           </cell>
           <cell r="H164" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I164">
-            <v>36222.829999999914</v>
+            <v>26870.565000000497</v>
           </cell>
         </row>
         <row r="165">
@@ -3802,13 +3793,13 @@
             <v>78750</v>
           </cell>
           <cell r="F165">
-            <v>53099.140000000007</v>
+            <v>135944.54999999996</v>
           </cell>
           <cell r="H165" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I165">
-            <v>25650.859999999993</v>
+            <v>12805.450000000041</v>
           </cell>
         </row>
         <row r="166">
@@ -3816,13 +3807,13 @@
             <v>122400</v>
           </cell>
           <cell r="F166">
-            <v>81243.350000000093</v>
+            <v>211937.01999999859</v>
           </cell>
           <cell r="H166" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I166">
-            <v>41156.649999999907</v>
+            <v>19262.980000001407</v>
           </cell>
         </row>
         <row r="167">
@@ -3844,13 +3835,13 @@
             <v>26100</v>
           </cell>
           <cell r="F168">
-            <v>15939.879999999988</v>
+            <v>39507.460000000057</v>
           </cell>
           <cell r="H168" t="str">
-            <v>D</v>
+            <v>C</v>
           </cell>
           <cell r="I168">
-            <v>10160.120000000012</v>
+            <v>1092.5399999999427</v>
           </cell>
         </row>
         <row r="169">
@@ -3858,13 +3849,13 @@
             <v>43200</v>
           </cell>
           <cell r="F169">
-            <v>25865.750000000011</v>
+            <v>62260.590000000026</v>
           </cell>
           <cell r="H169" t="str">
-            <v>D</v>
+            <v>C</v>
           </cell>
           <cell r="I169">
-            <v>17334.249999999989</v>
+            <v>4939.4099999999744</v>
           </cell>
         </row>
         <row r="170">
@@ -3872,13 +3863,13 @@
             <v>31725</v>
           </cell>
           <cell r="F170">
-            <v>19043.580000000002</v>
+            <v>48786.559999999998</v>
           </cell>
           <cell r="H170" t="str">
-            <v>D</v>
+            <v>C</v>
           </cell>
           <cell r="I170">
-            <v>12681.419999999998</v>
+            <v>563.44000000000233</v>
           </cell>
         </row>
         <row r="171">
@@ -3886,13 +3877,13 @@
             <v>37800</v>
           </cell>
           <cell r="F171">
-            <v>28099.500000000029</v>
+            <v>71931.839999999822</v>
           </cell>
           <cell r="H171" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I171">
-            <v>9700.4999999999709</v>
+            <v>12068.160000000178</v>
           </cell>
         </row>
         <row r="172">
@@ -3900,13 +3891,13 @@
             <v>63900</v>
           </cell>
           <cell r="F172">
-            <v>44023.619999999988</v>
+            <v>107918.3099999995</v>
           </cell>
           <cell r="H172" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I172">
-            <v>19876.380000000012</v>
+            <v>12781.690000000497</v>
           </cell>
         </row>
         <row r="173">
@@ -3914,13 +3905,13 @@
             <v>76050</v>
           </cell>
           <cell r="F173">
-            <v>48456.710000000006</v>
+            <v>130217.75999999982</v>
           </cell>
           <cell r="H173" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I173">
-            <v>27593.289999999994</v>
+            <v>13432.24000000018</v>
           </cell>
         </row>
         <row r="174">
@@ -3928,13 +3919,13 @@
             <v>121500</v>
           </cell>
           <cell r="F174">
-            <v>89009.680000000051</v>
+            <v>215409.78999999963</v>
           </cell>
           <cell r="H174" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I174">
-            <v>32490.319999999949</v>
+            <v>14090.21000000037</v>
           </cell>
         </row>
         <row r="175">
@@ -3942,13 +3933,13 @@
             <v>42975</v>
           </cell>
           <cell r="F175">
-            <v>18272.769999999997</v>
+            <v>45154.940000000046</v>
           </cell>
           <cell r="H175" t="str">
-            <v>D</v>
+            <v>C</v>
           </cell>
           <cell r="I175">
-            <v>24702.230000000003</v>
+            <v>21695.059999999954</v>
           </cell>
         </row>
         <row r="176">
@@ -3956,13 +3947,13 @@
             <v>97875</v>
           </cell>
           <cell r="F176">
-            <v>32493.730000000003</v>
+            <v>122031.32999999971</v>
           </cell>
           <cell r="H176" t="str">
-            <v>D</v>
+            <v>C</v>
           </cell>
           <cell r="I176">
-            <v>65381.27</v>
+            <v>30218.670000000289</v>
           </cell>
         </row>
         <row r="177">
@@ -3970,10 +3961,10 @@
             <v>1341000</v>
           </cell>
           <cell r="F177">
-            <v>883047.40000000037</v>
+            <v>2185106.5899999961</v>
           </cell>
           <cell r="I177">
-            <v>457952.59999999945</v>
+            <v>266668.41000000358</v>
           </cell>
         </row>
       </sheetData>
@@ -4853,19 +4844,19 @@
       </c>
       <c r="AN3" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI3,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>27951.950000000019</v>
+        <v>59228.230000000018</v>
       </c>
       <c r="AO3" s="26" t="str" cm="1">
         <f t="array" ref="AO3">_xlfn.IFS(AN3&gt;=AJ3,"A",AN3&gt;=AK3,"B",AN3&gt;=AL3,"C",AN3&gt;=AM3,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>D</v>
       </c>
       <c r="AP3" s="26" t="str" cm="1">
         <f t="array" ref="AP3">_xlfn.IFS(AO3="NÃO ATINGIDO","D",AO3="D","C",AO3="C","B",AO3="B","A",AO3="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="AQ3" s="25" cm="1">
         <f t="array" ref="AQ3">_xlfn.IFS(AP3="D",MAX(AM3-AN3,0),AP3="C",MAX(AL3-AN3,0),AP3="B",MAX(AK3-AN3,0),AP3="A",MAX(AJ3-AN3,0),AP3="OBJETIVO ALCANÇADO",0)</f>
-        <v>11648.049999999981</v>
+        <v>2371.769999999975</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -4886,7 +4877,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>300010</v>
+        <v>300470</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -4933,19 +4924,19 @@
       </c>
       <c r="AD4" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y4,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$M:$M,0),0)</f>
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="AE4" s="31" t="str" cm="1">
         <f t="array" ref="AE4">_xlfn.IFS(AD4&gt;=Z4,"A",AD4&gt;=AA4,"B",AD4&gt;=AB4,"C",AD4&gt;=AC4,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AF4" s="31" t="str" cm="1">
         <f t="array" ref="AF4">_xlfn.IFS(AE4="NÃO ATINGIDO","D",AE4="D","C",AE4="C","B",AE4="B","A",AE4="A","OBJETIVO ALCANÇADO")</f>
-        <v>C</v>
+        <v>A</v>
       </c>
       <c r="AG4" s="31" cm="1">
         <f t="array" ref="AG4">_xlfn.IFS(AF4="D",MAX(AC4-AD4,0),AF4="C",MAX(AB4-AD4,0),AF4="B",MAX(AA4-AD4,0),AF4="A",MAX(Z4-AD4,0),AF4="OBJETIVO ALCANÇADO",0)</f>
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="AI4" t="s">
         <v>24</v>
@@ -4968,19 +4959,19 @@
       </c>
       <c r="AN4" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI4,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>24446.020000000004</v>
+        <v>58769.760000000009</v>
       </c>
       <c r="AO4" s="26" t="str" cm="1">
         <f t="array" ref="AO4">_xlfn.IFS(AN4&gt;=AJ4,"A",AN4&gt;=AK4,"B",AN4&gt;=AL4,"C",AN4&gt;=AM4,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP4" s="26" t="str" cm="1">
         <f t="array" ref="AP4">_xlfn.IFS(AO4="NÃO ATINGIDO","D",AO4="D","C",AO4="C","B",AO4="B","A",AO4="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ4" s="25" cm="1">
         <f t="array" ref="AQ4">_xlfn.IFS(AP4="D",MAX(AM4-AN4,0),AP4="C",MAX(AL4-AN4,0),AP4="B",MAX(AK4-AN4,0),AP4="A",MAX(AJ4-AN4,0),AP4="OBJETIVO ALCANÇADO",0)</f>
-        <v>11103.979999999996</v>
+        <v>8380.2399999999907</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -4990,7 +4981,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>1561775.3300000003</v>
+        <v>3960015.8499999964</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -5001,7 +4992,7 @@
       </c>
       <c r="I5" s="7">
         <f ca="1">SUM(J10:J27)</f>
-        <v>89620.659999999974</v>
+        <v>2185106.5899999966</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -5023,7 +5014,7 @@
       </c>
       <c r="U5" s="4">
         <f ca="1">SUM(V10:V26)</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -5083,19 +5074,19 @@
       </c>
       <c r="AN5" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI5,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>117001.94999999997</v>
+        <v>272619.34999999963</v>
       </c>
       <c r="AO5" s="26" t="str" cm="1">
         <f t="array" ref="AO5">_xlfn.IFS(AN5&gt;=AJ5,"A",AN5&gt;=AK5,"B",AN5&gt;=AL5,"C",AN5&gt;=AM5,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP5" s="26" t="str" cm="1">
         <f t="array" ref="AP5">_xlfn.IFS(AO5="NÃO ATINGIDO","D",AO5="D","C",AO5="C","B",AO5="B","A",AO5="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ5" s="25" cm="1">
         <f t="array" ref="AQ5">_xlfn.IFS(AP5="D",MAX(AM5-AN5,0),AP5="C",MAX(AL5-AN5,0),AP5="B",MAX(AK5-AN5,0),AP5="A",MAX(AJ5-AN5,0),AP5="OBJETIVO ALCANÇADO",0)</f>
-        <v>38248.050000000032</v>
+        <v>20630.650000000373</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
@@ -5105,7 +5096,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>4469224.67</v>
+        <v>2070984.1500000036</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -5116,7 +5107,7 @@
       </c>
       <c r="I6" s="7">
         <f ca="1">I4-I5</f>
-        <v>210389.34000000003</v>
+        <v>-1884636.5899999966</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -5138,7 +5129,7 @@
       </c>
       <c r="U6" s="4">
         <f ca="1">U4-U5</f>
-        <v>460</v>
+        <v>560</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -5198,19 +5189,19 @@
       </c>
       <c r="AN6" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI6,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>114216.91000000018</v>
+        <v>251412.51500000042</v>
       </c>
       <c r="AO6" s="26" t="str" cm="1">
         <f t="array" ref="AO6">_xlfn.IFS(AN6&gt;=AJ6,"A",AN6&gt;=AK6,"B",AN6&gt;=AL6,"C",AN6&gt;=AM6,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP6" s="26" t="str" cm="1">
         <f t="array" ref="AP6">_xlfn.IFS(AO6="NÃO ATINGIDO","D",AO6="D","C",AO6="C","B",AO6="B","A",AO6="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ6" s="25" cm="1">
         <f t="array" ref="AQ6">_xlfn.IFS(AP6="D",MAX(AM6-AN6,0),AP6="C",MAX(AL6-AN6,0),AP6="B",MAX(AK6-AN6,0),AP6="A",MAX(AJ6-AN6,0),AP6="OBJETIVO ALCANÇADO",0)</f>
-        <v>34958.089999999822</v>
+        <v>30362.484999999579</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
@@ -5220,7 +5211,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.25895793898192676</v>
+        <v>0.65661015586138227</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -5231,7 +5222,7 @@
       </c>
       <c r="I7" s="3">
         <f ca="1">1-(I6/I4)</f>
-        <v>0.29872557581413939</v>
+        <v>7.2722953705860709</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -5253,7 +5244,7 @@
       </c>
       <c r="U7" s="3">
         <f ca="1">1-(U6/U4)</f>
-        <v>0.1785714285714286</v>
+        <v>0</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -5313,19 +5304,19 @@
       </c>
       <c r="AN7" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI7,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>87405.690000000031</v>
+        <v>203747.14999999964</v>
       </c>
       <c r="AO7" s="26" t="str" cm="1">
         <f t="array" ref="AO7">_xlfn.IFS(AN7&gt;=AJ7,"A",AN7&gt;=AK7,"B",AN7&gt;=AL7,"C",AN7&gt;=AM7,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP7" s="26" t="str" cm="1">
         <f t="array" ref="AP7">_xlfn.IFS(AO7="NÃO ATINGIDO","D",AO7="D","C",AO7="C","B",AO7="B","A",AO7="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ7" s="25" cm="1">
         <f t="array" ref="AQ7">_xlfn.IFS(AP7="D",MAX(AM7-AN7,0),AP7="C",MAX(AL7-AN7,0),AP7="B",MAX(AK7-AN7,0),AP7="A",MAX(AJ7-AN7,0),AP7="OBJETIVO ALCANÇADO",0)</f>
-        <v>39044.309999999969</v>
+        <v>35102.850000000355</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
@@ -5407,19 +5398,19 @@
       </c>
       <c r="AN8" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI8,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>56477.170000000086</v>
+        <v>148229.4349999995</v>
       </c>
       <c r="AO8" s="26" t="str" cm="1">
         <f t="array" ref="AO8">_xlfn.IFS(AN8&gt;=AJ8,"A",AN8&gt;=AK8,"B",AN8&gt;=AL8,"C",AN8&gt;=AM8,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP8" s="26" t="str" cm="1">
         <f t="array" ref="AP8">_xlfn.IFS(AO8="NÃO ATINGIDO","D",AO8="D","C",AO8="C","B",AO8="B","A",AO8="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ8" s="25" cm="1">
         <f t="array" ref="AQ8">_xlfn.IFS(AP8="D",MAX(AM8-AN8,0),AP8="C",MAX(AL8-AN8,0),AP8="B",MAX(AK8-AN8,0),AP8="A",MAX(AJ8-AN8,0),AP8="OBJETIVO ALCANÇADO",0)</f>
-        <v>36222.829999999914</v>
+        <v>26870.565000000497</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -5458,7 +5449,7 @@
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
@@ -5534,19 +5525,19 @@
       </c>
       <c r="AN9" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI9,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>53099.140000000007</v>
+        <v>135944.54999999996</v>
       </c>
       <c r="AO9" s="26" t="str" cm="1">
         <f t="array" ref="AO9">_xlfn.IFS(AN9&gt;=AJ9,"A",AN9&gt;=AK9,"B",AN9&gt;=AL9,"C",AN9&gt;=AM9,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP9" s="26" t="str" cm="1">
         <f t="array" ref="AP9">_xlfn.IFS(AO9="NÃO ATINGIDO","D",AO9="D","C",AO9="C","B",AO9="B","A",AO9="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ9" s="25" cm="1">
         <f t="array" ref="AQ9">_xlfn.IFS(AP9="D",MAX(AM9-AN9,0),AP9="C",MAX(AL9-AN9,0),AP9="B",MAX(AK9-AN9,0),AP9="A",MAX(AJ9-AN9,0),AP9="OBJETIVO ALCANÇADO",0)</f>
-        <v>25650.859999999993</v>
+        <v>12805.450000000041</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.25">
@@ -5562,11 +5553,11 @@
       </c>
       <c r="D10" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>19043.580000000002</v>
+        <v>48786.559999999998</v>
       </c>
       <c r="E10" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>51456.42</v>
+        <v>21713.440000000002</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="18" t="s">
@@ -5577,15 +5568,15 @@
       </c>
       <c r="I10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>28000</v>
+        <v>28040</v>
       </c>
       <c r="J10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13963.489999999998</v>
+        <v>251412.51500000042</v>
       </c>
       <c r="K10" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>14036.510000000002</v>
+        <v>-223372.51500000042</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -5678,19 +5669,19 @@
       </c>
       <c r="AN10" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>81243.350000000093</v>
+        <v>211937.01999999859</v>
       </c>
       <c r="AO10" s="26" t="str" cm="1">
         <f t="array" ref="AO10">_xlfn.IFS(AN10&gt;=AJ10,"A",AN10&gt;=AK10,"B",AN10&gt;=AL10,"C",AN10&gt;=AM10,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP10" s="26" t="str" cm="1">
         <f t="array" ref="AP10">_xlfn.IFS(AO10="NÃO ATINGIDO","D",AO10="D","C",AO10="C","B",AO10="B","A",AO10="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ10" s="25" cm="1">
         <f t="array" ref="AQ10">_xlfn.IFS(AP10="D",MAX(AM10-AN10,0),AP10="C",MAX(AL10-AN10,0),AP10="B",MAX(AK10-AN10,0),AP10="A",MAX(AJ10-AN10,0),AP10="OBJETIVO ALCANÇADO",0)</f>
-        <v>41156.649999999907</v>
+        <v>19262.980000001407</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.25">
@@ -5706,11 +5697,11 @@
       </c>
       <c r="D11" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>117001.94999999997</v>
+        <v>272619.34999999963</v>
       </c>
       <c r="E11" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>227998.05000000005</v>
+        <v>72380.650000000373</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="18" t="s">
@@ -5725,11 +5716,11 @@
       </c>
       <c r="J11" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5135.0499999999984</v>
+        <v>211937.01999999859</v>
       </c>
       <c r="K11" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>19864.95</v>
+        <v>-186937.01999999859</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -5763,11 +5754,11 @@
       </c>
       <c r="V11" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W11" s="17">
         <f t="shared" ref="W11:W20" ca="1" si="0">U11-V11</f>
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="Y11" s="32" t="s">
         <v>12</v>
@@ -5853,11 +5844,11 @@
       </c>
       <c r="D12" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>324.10000000000002</v>
+        <v>0</v>
       </c>
       <c r="E12" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>-324.10000000000002</v>
+        <v>0</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="18" t="s">
@@ -5868,15 +5859,15 @@
       </c>
       <c r="I12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>14510</v>
+        <v>14810</v>
       </c>
       <c r="J12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2919.1</v>
+        <v>107918.3099999995</v>
       </c>
       <c r="K12" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11590.9</v>
+        <v>-93108.309999999503</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -5910,11 +5901,11 @@
       </c>
       <c r="V12" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W12" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="Y12" s="33" t="s">
         <v>23</v>
@@ -5972,19 +5963,19 @@
       </c>
       <c r="AN12" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI12,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>15939.879999999988</v>
+        <v>39507.460000000057</v>
       </c>
       <c r="AO12" s="26" t="str" cm="1">
         <f t="array" ref="AO12">_xlfn.IFS(AN12&gt;=AJ12,"A",AN12&gt;=AK12,"B",AN12&gt;=AL12,"C",AN12&gt;=AM12,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>D</v>
       </c>
       <c r="AP12" s="26" t="str" cm="1">
         <f t="array" ref="AP12">_xlfn.IFS(AO12="NÃO ATINGIDO","D",AO12="D","C",AO12="C","B",AO12="B","A",AO12="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="AQ12" s="25" cm="1">
         <f t="array" ref="AQ12">_xlfn.IFS(AP12="D",MAX(AM12-AN12,0),AP12="C",MAX(AL12-AN12,0),AP12="B",MAX(AK12-AN12,0),AP12="A",MAX(AJ12-AN12,0),AP12="OBJETIVO ALCANÇADO",0)</f>
-        <v>10160.120000000012</v>
+        <v>1092.5399999999427</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.25">
@@ -6000,11 +5991,11 @@
       </c>
       <c r="D13" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>25865.750000000011</v>
+        <v>62260.590000000026</v>
       </c>
       <c r="E13" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>70134.249999999985</v>
+        <v>33739.409999999974</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="18" t="s">
@@ -6015,15 +6006,15 @@
       </c>
       <c r="I13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>24000</v>
+        <v>25000</v>
       </c>
       <c r="J13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>15594.409999999996</v>
+        <v>215409.78999999963</v>
       </c>
       <c r="K13" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8405.5900000000038</v>
+        <v>-190409.78999999963</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -6057,11 +6048,11 @@
       </c>
       <c r="V13" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="W13" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="Y13" s="32" t="s">
         <v>9</v>
@@ -6119,19 +6110,19 @@
       </c>
       <c r="AN13" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>25865.750000000011</v>
+        <v>62260.590000000026</v>
       </c>
       <c r="AO13" s="26" t="str" cm="1">
         <f t="array" ref="AO13">_xlfn.IFS(AN13&gt;=AJ13,"A",AN13&gt;=AK13,"B",AN13&gt;=AL13,"C",AN13&gt;=AM13,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>D</v>
       </c>
       <c r="AP13" s="26" t="str" cm="1">
         <f t="array" ref="AP13">_xlfn.IFS(AO13="NÃO ATINGIDO","D",AO13="D","C",AO13="C","B",AO13="B","A",AO13="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="AQ13" s="25" cm="1">
         <f t="array" ref="AQ13">_xlfn.IFS(AP13="D",MAX(AM13-AN13,0),AP13="C",MAX(AL13-AN13,0),AP13="B",MAX(AK13-AN13,0),AP13="A",MAX(AJ13-AN13,0),AP13="OBJETIVO ALCANÇADO",0)</f>
-        <v>17334.249999999989</v>
+        <v>4939.4099999999744</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.25">
@@ -6147,11 +6138,11 @@
       </c>
       <c r="D14" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>87405.690000000031</v>
+        <v>203747.14999999964</v>
       </c>
       <c r="E14" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>193594.30999999997</v>
+        <v>77252.850000000355</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="18" t="s">
@@ -6162,15 +6153,15 @@
       </c>
       <c r="I14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>19770</v>
+        <v>20630</v>
       </c>
       <c r="J14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1402.54</v>
+        <v>122031.32999999971</v>
       </c>
       <c r="K14" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>18367.46</v>
+        <v>-101401.32999999971</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -6204,11 +6195,11 @@
       </c>
       <c r="V14" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W14" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="Y14" s="33" t="s">
         <v>7</v>
@@ -6266,19 +6257,19 @@
       </c>
       <c r="AN14" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>19043.580000000002</v>
+        <v>48786.559999999998</v>
       </c>
       <c r="AO14" s="26" t="str" cm="1">
         <f t="array" ref="AO14">_xlfn.IFS(AN14&gt;=AJ14,"A",AN14&gt;=AK14,"B",AN14&gt;=AL14,"C",AN14&gt;=AM14,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>D</v>
       </c>
       <c r="AP14" s="26" t="str" cm="1">
         <f t="array" ref="AP14">_xlfn.IFS(AO14="NÃO ATINGIDO","D",AO14="D","C",AO14="C","B",AO14="B","A",AO14="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="AQ14" s="25" cm="1">
         <f t="array" ref="AQ14">_xlfn.IFS(AP14="D",MAX(AM14-AN14,0),AP14="C",MAX(AL14-AN14,0),AP14="B",MAX(AK14-AN14,0),AP14="A",MAX(AJ14-AN14,0),AP14="OBJETIVO ALCANÇADO",0)</f>
-        <v>12681.419999999998</v>
+        <v>563.44000000000233</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.25">
@@ -6294,11 +6285,11 @@
       </c>
       <c r="D15" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>28099.500000000029</v>
+        <v>71931.839999999822</v>
       </c>
       <c r="E15" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>55900.499999999971</v>
+        <v>12068.160000000178</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="18" t="s">
@@ -6309,15 +6300,15 @@
       </c>
       <c r="I15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>31000</v>
+        <v>32000</v>
       </c>
       <c r="J15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>11533.52</v>
+        <v>272619.34999999963</v>
       </c>
       <c r="K15" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>19466.48</v>
+        <v>-240619.34999999963</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -6413,19 +6404,19 @@
       </c>
       <c r="AN15" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>28099.500000000029</v>
+        <v>71931.839999999822</v>
       </c>
       <c r="AO15" s="26" t="str" cm="1">
         <f t="array" ref="AO15">_xlfn.IFS(AN15&gt;=AJ15,"A",AN15&gt;=AK15,"B",AN15&gt;=AL15,"C",AN15&gt;=AM15,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP15" s="26" t="str" cm="1">
         <f t="array" ref="AP15">_xlfn.IFS(AO15="NÃO ATINGIDO","D",AO15="D","C",AO15="C","B",AO15="B","A",AO15="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ15" s="25" cm="1">
         <f t="array" ref="AQ15">_xlfn.IFS(AP15="D",MAX(AM15-AN15,0),AP15="C",MAX(AL15-AN15,0),AP15="B",MAX(AK15-AN15,0),AP15="A",MAX(AJ15-AN15,0),AP15="OBJETIVO ALCANÇADO",0)</f>
-        <v>9700.4999999999709</v>
+        <v>12068.160000000178</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.25">
@@ -6441,11 +6432,11 @@
       </c>
       <c r="D16" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>90046.700000000012</v>
+        <v>194941.35</v>
       </c>
       <c r="E16" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>259953.3</v>
+        <v>155058.65</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="18" t="s">
@@ -6456,15 +6447,15 @@
       </c>
       <c r="I16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>19620</v>
+        <v>18000</v>
       </c>
       <c r="J16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2159.1999999999998</v>
+        <v>135944.54999999996</v>
       </c>
       <c r="K16" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>17460.8</v>
+        <v>-117944.54999999996</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -6560,19 +6551,19 @@
       </c>
       <c r="AN16" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>44023.619999999988</v>
+        <v>107918.3099999995</v>
       </c>
       <c r="AO16" s="26" t="str" cm="1">
         <f t="array" ref="AO16">_xlfn.IFS(AN16&gt;=AJ16,"A",AN16&gt;=AK16,"B",AN16&gt;=AL16,"C",AN16&gt;=AM16,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP16" s="26" t="str" cm="1">
         <f t="array" ref="AP16">_xlfn.IFS(AO16="NÃO ATINGIDO","D",AO16="D","C",AO16="C","B",AO16="B","A",AO16="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ16" s="25" cm="1">
         <f t="array" ref="AQ16">_xlfn.IFS(AP16="D",MAX(AM16-AN16,0),AP16="C",MAX(AL16-AN16,0),AP16="B",MAX(AK16-AN16,0),AP16="A",MAX(AJ16-AN16,0),AP16="OBJETIVO ALCANÇADO",0)</f>
-        <v>19876.380000000012</v>
+        <v>12781.690000000497</v>
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.25">
@@ -6588,11 +6579,11 @@
       </c>
       <c r="D17" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>104355.99000000003</v>
+        <v>350628.99999999953</v>
       </c>
       <c r="E17" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>395644.00999999995</v>
+        <v>149371.00000000047</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="18" t="s">
@@ -6603,15 +6594,15 @@
       </c>
       <c r="I17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>10110</v>
+        <v>9790</v>
       </c>
       <c r="J17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2549.5500000000002</v>
+        <v>45154.940000000046</v>
       </c>
       <c r="K17" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7560.45</v>
+        <v>-35364.940000000046</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -6645,11 +6636,11 @@
       </c>
       <c r="V17" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="W17" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="Y17" s="32" t="s">
         <v>14</v>
@@ -6707,19 +6698,19 @@
       </c>
       <c r="AN17" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>48456.710000000006</v>
+        <v>130217.75999999982</v>
       </c>
       <c r="AO17" s="26" t="str" cm="1">
         <f t="array" ref="AO17">_xlfn.IFS(AN17&gt;=AJ17,"A",AN17&gt;=AK17,"B",AN17&gt;=AL17,"C",AN17&gt;=AM17,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP17" s="26" t="str" cm="1">
         <f t="array" ref="AP17">_xlfn.IFS(AO17="NÃO ATINGIDO","D",AO17="D","C",AO17="C","B",AO17="B","A",AO17="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ17" s="25" cm="1">
         <f t="array" ref="AQ17">_xlfn.IFS(AP17="D",MAX(AM17-AN17,0),AP17="C",MAX(AL17-AN17,0),AP17="B",MAX(AK17-AN17,0),AP17="A",MAX(AJ17-AN17,0),AP17="OBJETIVO ALCANÇADO",0)</f>
-        <v>27593.289999999994</v>
+        <v>13432.24000000018</v>
       </c>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.25">
@@ -6735,11 +6726,11 @@
       </c>
       <c r="D18" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>284976.00000000006</v>
+        <v>560129.58000000042</v>
       </c>
       <c r="E18" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>695024</v>
+        <v>419870.41999999958</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="18" t="s">
@@ -6841,19 +6832,19 @@
       </c>
       <c r="AN18" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>89009.680000000051</v>
+        <v>215409.78999999963</v>
       </c>
       <c r="AO18" s="26" t="str" cm="1">
         <f t="array" ref="AO18">_xlfn.IFS(AN18&gt;=AJ18,"A",AN18&gt;=AK18,"B",AN18&gt;=AL18,"C",AN18&gt;=AM18,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP18" s="26" t="str" cm="1">
         <f t="array" ref="AP18">_xlfn.IFS(AO18="NÃO ATINGIDO","D",AO18="D","C",AO18="C","B",AO18="B","A",AO18="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ18" s="25" cm="1">
         <f t="array" ref="AQ18">_xlfn.IFS(AP18="D",MAX(AM18-AN18,0),AP18="C",MAX(AL18-AN18,0),AP18="B",MAX(AK18-AN18,0),AP18="A",MAX(AJ18-AN18,0),AP18="OBJETIVO ALCANÇADO",0)</f>
-        <v>32490.319999999949</v>
+        <v>14090.21000000037</v>
       </c>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.25">
@@ -6869,11 +6860,11 @@
       </c>
       <c r="D19" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>10406.4</v>
+        <v>45062.200000000004</v>
       </c>
       <c r="E19" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>139593.60000000001</v>
+        <v>104937.79999999999</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="18" t="s">
@@ -6884,15 +6875,15 @@
       </c>
       <c r="I19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>19890</v>
+        <v>17000</v>
       </c>
       <c r="J19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>988.43000000000006</v>
+        <v>148229.4349999995</v>
       </c>
       <c r="K19" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>18901.57</v>
+        <v>-131229.4349999995</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -6909,11 +6900,11 @@
       </c>
       <c r="V19" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="W19" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="Y19" s="32" t="s">
         <v>16</v>
@@ -6971,19 +6962,19 @@
       </c>
       <c r="AN19" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>18272.769999999997</v>
+        <v>45154.940000000046</v>
       </c>
       <c r="AO19" s="26" t="str" cm="1">
         <f t="array" ref="AO19">_xlfn.IFS(AN19&gt;=AJ19,"A",AN19&gt;=AK19,"B",AN19&gt;=AL19,"C",AN19&gt;=AM19,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>D</v>
       </c>
       <c r="AP19" s="26" t="str" cm="1">
         <f t="array" ref="AP19">_xlfn.IFS(AO19="NÃO ATINGIDO","D",AO19="D","C",AO19="C","B",AO19="B","A",AO19="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="AQ19" s="25" cm="1">
         <f t="array" ref="AQ19">_xlfn.IFS(AP19="D",MAX(AM19-AN19,0),AP19="C",MAX(AL19-AN19,0),AP19="B",MAX(AK19-AN19,0),AP19="A",MAX(AJ19-AN19,0),AP19="OBJETIVO ALCANÇADO",0)</f>
-        <v>24702.230000000003</v>
+        <v>21695.059999999954</v>
       </c>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.25">
@@ -6999,11 +6990,11 @@
       </c>
       <c r="D20" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>76109.040000000023</v>
+        <v>288574.25999999995</v>
       </c>
       <c r="E20" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>513890.95999999996</v>
+        <v>301425.74000000005</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="18" t="s">
@@ -7014,15 +7005,15 @@
       </c>
       <c r="I20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>25000</v>
+        <v>24730</v>
       </c>
       <c r="J20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10562.029999999999</v>
+        <v>203747.14999999964</v>
       </c>
       <c r="K20" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>14437.970000000001</v>
+        <v>-179017.14999999964</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -7051,11 +7042,11 @@
       </c>
       <c r="V20" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="W20" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="Y20" s="33" t="s">
         <v>15</v>
@@ -7113,19 +7104,19 @@
       </c>
       <c r="AN20" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>32493.730000000003</v>
+        <v>122031.32999999971</v>
       </c>
       <c r="AO20" s="26" t="str" cm="1">
         <f t="array" ref="AO20">_xlfn.IFS(AN20&gt;=AJ20,"A",AN20&gt;=AK20,"B",AN20&gt;=AL20,"C",AN20&gt;=AM20,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>D</v>
       </c>
       <c r="AP20" s="26" t="str" cm="1">
         <f t="array" ref="AP20">_xlfn.IFS(AO20="NÃO ATINGIDO","D",AO20="D","C",AO20="C","B",AO20="B","A",AO20="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="AQ20" s="25" cm="1">
         <f t="array" ref="AQ20">_xlfn.IFS(AP20="D",MAX(AM20-AN20,0),AP20="C",MAX(AL20-AN20,0),AP20="B",MAX(AK20-AN20,0),AP20="A",MAX(AJ20-AN20,0),AP20="OBJETIVO ALCANÇADO",0)</f>
-        <v>65381.27</v>
+        <v>30218.670000000289</v>
       </c>
     </row>
     <row r="21" spans="1:43" x14ac:dyDescent="0.25">
@@ -7141,11 +7132,11 @@
       </c>
       <c r="D21" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>112434.5800000001</v>
+        <v>334703.23000000004</v>
       </c>
       <c r="E21" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>367565.41999999993</v>
+        <v>145296.76999999996</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="18" t="s">
@@ -7156,15 +7147,15 @@
       </c>
       <c r="I21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>5700</v>
+        <v>5820</v>
       </c>
       <c r="J21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2244.54</v>
+        <v>71931.839999999822</v>
       </c>
       <c r="K21" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3455.46</v>
+        <v>-66111.839999999822</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -7196,11 +7187,11 @@
       </c>
       <c r="V21" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W21" s="17">
         <f t="shared" ref="W21:W26" ca="1" si="1">U21-V21</f>
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="Y21" s="36" t="s">
         <v>60</v>
@@ -7223,13 +7214,13 @@
       </c>
       <c r="AD21" s="37">
         <f>SUBTOTAL(109,Planilha1!$AD$3:$AD$20)</f>
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="AE21" s="37"/>
       <c r="AF21" s="37"/>
       <c r="AG21" s="38">
         <f>SUBTOTAL(109,Planilha1!$AG$3:$AG$20)</f>
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="AI21" t="s">
         <v>60</v>
@@ -7252,13 +7243,13 @@
       </c>
       <c r="AN21" s="26">
         <f>SUBTOTAL(109,Tabela817[ATINGIDO])</f>
-        <v>883047.40000000037</v>
+        <v>2185106.5899999961</v>
       </c>
       <c r="AO21" s="4"/>
       <c r="AP21" s="4"/>
       <c r="AQ21" s="27">
         <f>SUBTOTAL(109,Tabela817[FALTA])</f>
-        <v>457952.59999999945</v>
+        <v>266668.41000000358</v>
       </c>
     </row>
     <row r="22" spans="1:43" x14ac:dyDescent="0.25">
@@ -7293,11 +7284,11 @@
       </c>
       <c r="J22" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4973.12</v>
+        <v>130217.75999999982</v>
       </c>
       <c r="K22" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>16026.880000000001</v>
+        <v>-109217.75999999982</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -7310,11 +7301,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>100872.79000000004</v>
+        <v>102026.29000000004</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>625317.68619047618</v>
+        <v>624164.18619047618</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="17" t="s">
@@ -7329,11 +7320,11 @@
       </c>
       <c r="V22" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="W22" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:43" x14ac:dyDescent="0.25">
@@ -7349,11 +7340,11 @@
       </c>
       <c r="D23" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>56477.170000000086</v>
+        <v>148229.4349999995</v>
       </c>
       <c r="E23" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>149522.8299999999</v>
+        <v>57770.565000000497</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="18" t="s">
@@ -7364,15 +7355,15 @@
       </c>
       <c r="I23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>15530</v>
+        <v>15850</v>
       </c>
       <c r="J23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4577.72</v>
+        <v>62260.590000000026</v>
       </c>
       <c r="K23" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10952.279999999999</v>
+        <v>-46410.590000000026</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -7385,11 +7376,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>0</v>
+        <v>190257.24000000017</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>580952.38095238095</v>
+        <v>390695.14095238078</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="17" t="s">
@@ -7404,11 +7395,11 @@
       </c>
       <c r="V23" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="W23" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:43" x14ac:dyDescent="0.25">
@@ -7424,11 +7415,11 @@
       </c>
       <c r="D24" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>48456.710000000006</v>
+        <v>130217.75999999982</v>
       </c>
       <c r="E24" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>120543.29</v>
+        <v>38782.24000000018</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="18" t="s">
@@ -7439,15 +7430,15 @@
       </c>
       <c r="I24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>10850</v>
+        <v>11080</v>
       </c>
       <c r="J24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2619.7000000000003</v>
+        <v>58769.760000000009</v>
       </c>
       <c r="K24" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8230.2999999999993</v>
+        <v>-47689.760000000009</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -7460,11 +7451,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>0</v>
+        <v>54862.269999999917</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>726190.47619047621</v>
+        <v>671328.20619047631</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="17" t="s">
@@ -7479,11 +7470,11 @@
       </c>
       <c r="V24" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W24" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:43" x14ac:dyDescent="0.25">
@@ -7499,11 +7490,11 @@
       </c>
       <c r="D25" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>32493.730000000003</v>
+        <v>122031.32999999971</v>
       </c>
       <c r="E25" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>185006.27</v>
+        <v>95468.670000000289</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="18" t="s">
@@ -7514,15 +7505,15 @@
       </c>
       <c r="I25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>15300</v>
+        <v>15790</v>
       </c>
       <c r="J25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5642.74</v>
+        <v>59228.230000000018</v>
       </c>
       <c r="K25" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9657.26</v>
+        <v>-43438.230000000018</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -7554,11 +7545,11 @@
       </c>
       <c r="V25" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W25" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:43" x14ac:dyDescent="0.25">
@@ -7574,11 +7565,11 @@
       </c>
       <c r="D26" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>18272.769999999997</v>
+        <v>45154.940000000046</v>
       </c>
       <c r="E26" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>77227.23000000001</v>
+        <v>50345.059999999954</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="18" t="s">
@@ -7589,15 +7580,15 @@
       </c>
       <c r="I26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>8980</v>
+        <v>10060</v>
       </c>
       <c r="J26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1484.7000000000003</v>
+        <v>39507.460000000057</v>
       </c>
       <c r="K26" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7495.2999999999993</v>
+        <v>-29447.460000000057</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -7618,11 +7609,11 @@
       </c>
       <c r="V26" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W26" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:43" x14ac:dyDescent="0.25">
@@ -7638,11 +7629,11 @@
       </c>
       <c r="D27" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>81243.350000000093</v>
+        <v>211937.01999999859</v>
       </c>
       <c r="E27" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>190756.64999999991</v>
+        <v>60062.980000001407</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="18" t="s">
@@ -7653,15 +7644,15 @@
       </c>
       <c r="I27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>5750</v>
+        <v>5870</v>
       </c>
       <c r="J27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1270.82</v>
+        <v>48786.559999999998</v>
       </c>
       <c r="K27" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4479.18</v>
+        <v>-42916.56</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -7684,11 +7675,11 @@
       </c>
       <c r="D28" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>114216.91000000018</v>
+        <v>251412.51500000042</v>
       </c>
       <c r="E28" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>217283.08999999982</v>
+        <v>80087.484999999579</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -7763,11 +7754,11 @@
       </c>
       <c r="D30" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>44023.619999999988</v>
+        <v>107918.3099999995</v>
       </c>
       <c r="E30" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>97976.38</v>
+        <v>34081.690000000497</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -7820,11 +7811,11 @@
       </c>
       <c r="D31" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>53099.140000000007</v>
+        <v>135944.54999999996</v>
       </c>
       <c r="E31" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>121900.85999999999</v>
+        <v>39055.450000000041</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -7837,11 +7828,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>120065.70999999995</v>
+        <v>119805.16999999987</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>163743.81380952382</v>
+        <v>164004.35380952392</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -7860,11 +7851,11 @@
       </c>
       <c r="V31" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[2]"),0)</f>
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="W31" s="6">
         <f t="shared" ref="W31:W33" si="2">U31-V31</f>
-        <v>54.333333333333343</v>
+        <v>55.333333333333343</v>
       </c>
     </row>
     <row r="32" spans="1:43" x14ac:dyDescent="0.25">
@@ -7880,11 +7871,11 @@
       </c>
       <c r="D32" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>89009.680000000051</v>
+        <v>215409.78999999963</v>
       </c>
       <c r="E32" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>180990.31999999995</v>
+        <v>54590.21000000037</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -7897,11 +7888,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>587944.82000000135</v>
+        <v>583783.27000000176</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="3">I32-J32</f>
-        <v>121578.98952380812</v>
+        <v>125740.5395238077</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -7940,11 +7931,11 @@
       </c>
       <c r="D33" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>27951.950000000019</v>
+        <v>59228.230000000018</v>
       </c>
       <c r="E33" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>60048.049999999981</v>
+        <v>28771.769999999982</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -7957,11 +7948,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>0</v>
+        <v>485447.22000000247</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="3"/>
-        <v>567619.04761904757</v>
+        <v>82171.8276190451</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -8000,11 +7991,11 @@
       </c>
       <c r="D34" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>15939.879999999988</v>
+        <v>39507.460000000057</v>
       </c>
       <c r="E34" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>42060.12000000001</v>
+        <v>18492.539999999943</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -8017,11 +8008,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>0</v>
+        <v>541962.97500000265</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="3"/>
-        <v>709523.80952380947</v>
+        <v>167560.83452380681</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -8060,11 +8051,11 @@
       </c>
       <c r="D35" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>24446.020000000004</v>
+        <v>58769.760000000009</v>
       </c>
       <c r="E35" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>54553.979999999996</v>
+        <v>20230.239999999991</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -8109,11 +8100,11 @@
       </c>
       <c r="D36" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>75.12</v>
+        <v>869.6400000000001</v>
       </c>
       <c r="E36" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>924.88</v>
+        <v>130.3599999999999</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -8220,11 +8211,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>163093.37999999971</v>
+        <v>162832.92999999959</v>
       </c>
       <c r="E40" s="7">
         <f>C40-D40</f>
-        <v>411287.57238095271</v>
+        <v>411548.02238095284</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -8256,11 +8247,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1398857.0399999972</v>
+        <v>1394652.559999998</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" ref="E41:E43" si="4">C41-D41</f>
-        <v>37095.34095238382</v>
+        <v>41299.820952383103</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -8292,11 +8283,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>0</v>
+        <v>1139532.6350000028</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="4"/>
-        <v>1148761.9047619049</v>
+        <v>9229.2697619020473</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -8328,11 +8319,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>0</v>
+        <v>1263493.1849999924</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="4"/>
-        <v>1435952.3809523811</v>
+        <v>172459.19595238869</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>